<commit_message>
Use CP names in event import template
</commit_message>
<xml_diff>
--- a/public/templates/events-import.xlsx
+++ b/public/templates/events-import.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="活动导入" sheetId="1" r:id="R1e2e94096a51434e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="填写说明" sheetId="2" r:id="R8515639d00464497"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="活动导入" sheetId="1" r:id="R6defe0a624d440f9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="填写说明" sheetId="2" r:id="R9bbc751da35a484a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -393,7 +393,7 @@
         <x:v>0.7916666666666666</x:v>
       </x:c>
       <x:c r="C3" s="5" t="str">
-        <x:v>Auau Thanaphum / Patji Jirachart / Ryujin Tinnapat / Save Worapong</x:v>
+        <x:v>AuAuSave / RyujinPatji</x:v>
       </x:c>
       <x:c r="D3" s="5" t="str">
         <x:v>Flex Talk电台</x:v>
@@ -4279,7 +4279,7 @@
         <x:v>艺人名称</x:v>
       </x:c>
       <x:c r="B3" s="2" t="str">
-        <x:v>多位艺人用 / 分隔。公司和艺人类别由后台资料自动带出；未匹配名称可先导入草稿再匹配。</x:v>
+        <x:v>CP 直接填写后台 CP 名称，不展开成员全名；多位艺人或 CP 用 / 分隔。公司和艺人类别由后台资料自动带出；未匹配名称可先导入草稿再匹配。</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="48" customHeight="1">

</xml_diff>

<commit_message>
Add event bulk management and source links
</commit_message>
<xml_diff>
--- a/public/templates/events-import.xlsx
+++ b/public/templates/events-import.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="活动导入" sheetId="1" r:id="R6defe0a624d440f9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="填写说明" sheetId="2" r:id="R9bbc751da35a484a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="活动导入" sheetId="1" r:id="R7d87dd5f411d44d4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="填写说明" sheetId="2" r:id="R261203150ae144a8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4234,7 +4234,7 @@
   </x:mergeCells>
   <x:dataValidations count="4">
     <x:dataValidation type="list" sqref="G3:G203">
-      <x:formula1>"演出舞台,影视宣传,站台活动,颁奖红毯,线上直播,其他"</x:formula1>
+      <x:formula1>"演出舞台,影视宣传,见面会/签售,发布会/记者会,站台活动,颁奖红毯,线上直播,其他"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="H3:H203">
       <x:formula1>"中国,泰国,其他国家或地区,线上"</x:formula1>

</xml_diff>